<commit_message>
V3: April 2026, new sequence files with new constraints and taks blocks read in condition files more flexibly
</commit_message>
<xml_diff>
--- a/sequences/TSRlearn_blockA.xlsx
+++ b/sequences/TSRlearn_blockA.xlsx
@@ -32,10 +32,10 @@
     <t>condFileretr</t>
   </si>
   <si>
-    <t>sequences/learning_blockA_fixed-middle-10_02.xlsx</t>
+    <t>sequences/learning_blockA_fixed-middle-10</t>
   </si>
   <si>
-    <t>sequences/retrieval_blockA_fixed-middle-10_02.xlsx</t>
+    <t>sequences/retrieval_blockA_fixed-middle-10</t>
   </si>
 </sst>
 </file>

</xml_diff>